<commit_message>
docs: update comp560 schedule spreadsheet
</commit_message>
<xml_diff>
--- a/comp560-schedule.xlsx
+++ b/comp560-schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp560-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F20C522-CAE9-412C-B73D-A853C09E65C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CBB5306-000C-4F94-99C9-17D012E37D27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="73">
   <si>
     <t>Marking period</t>
   </si>
@@ -225,6 +225,33 @@
   </si>
   <si>
     <t>updated 9/2/2026</t>
+  </si>
+  <si>
+    <t>honors projects</t>
+  </si>
+  <si>
+    <t>Mon 9/21</t>
+  </si>
+  <si>
+    <t>FRP</t>
+  </si>
+  <si>
+    <t>Mon 9/14</t>
+  </si>
+  <si>
+    <t>Mon 12/7</t>
+  </si>
+  <si>
+    <t>RR</t>
+  </si>
+  <si>
+    <t>Mon 11/30</t>
+  </si>
+  <si>
+    <t>complete draft of FRP</t>
+  </si>
+  <si>
+    <t>complete draft of RR</t>
   </si>
 </sst>
 </file>
@@ -293,7 +320,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -655,11 +682,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -750,30 +799,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -792,24 +847,34 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1117,7 +1182,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.28515625" style="6" customWidth="1"/>
@@ -1125,9 +1190,10 @@
     <col min="4" max="4" width="11" style="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.5703125" style="7" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="4" customFormat="1" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -1141,15 +1207,18 @@
       <c r="E1" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="43" t="s">
+      <c r="F1" s="53" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="53" t="s">
+      <c r="G1" s="37" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="50" t="s">
+      <c r="B2" s="43" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="15">
@@ -1157,11 +1226,12 @@
       </c>
       <c r="D2" s="16"/>
       <c r="E2" s="31"/>
-      <c r="F2" s="36"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="54"/>
-      <c r="B3" s="51"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="60"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="41"/>
+      <c r="B3" s="44"/>
       <c r="C3" s="3">
         <v>46267</v>
       </c>
@@ -1169,11 +1239,12 @@
       <c r="E3" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="37"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="54"/>
-      <c r="B4" s="52"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="61"/>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="41"/>
+      <c r="B4" s="45"/>
       <c r="C4" s="9">
         <v>46273</v>
       </c>
@@ -1181,11 +1252,12 @@
         <v>17</v>
       </c>
       <c r="E4" s="33"/>
-      <c r="F4" s="38"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="54"/>
-      <c r="B5" s="50" t="s">
+      <c r="F4" s="56"/>
+      <c r="G4" s="62"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="41"/>
+      <c r="B5" s="43" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="15">
@@ -1195,549 +1267,600 @@
       <c r="E5" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="36"/>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="54"/>
-      <c r="B6" s="52"/>
-      <c r="C6" s="9">
+      <c r="F5" s="54"/>
+      <c r="G5" s="60"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="41"/>
+      <c r="B6" s="44"/>
+      <c r="C6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="61" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="41"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="9">
         <f>C5+6</f>
         <v>46280</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D7" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="33"/>
-      <c r="F6" s="38"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="54"/>
-      <c r="B7" s="50" t="s">
+      <c r="E7" s="33"/>
+      <c r="F7" s="56"/>
+      <c r="G7" s="62"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="41"/>
+      <c r="B8" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C8" s="15">
         <f>C5+7</f>
         <v>46281</v>
       </c>
-      <c r="D7" s="18"/>
-      <c r="E7" s="31" t="s">
+      <c r="D8" s="18"/>
+      <c r="E8" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="36"/>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="55"/>
-      <c r="B8" s="52"/>
-      <c r="C8" s="9">
-        <f t="shared" ref="C8" si="0">C7+6</f>
+      <c r="F8" s="54"/>
+      <c r="G8" s="60"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="52"/>
+      <c r="B9" s="44"/>
+      <c r="C9" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="61" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="42"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="9">
+        <f t="shared" ref="C10" si="0">C8+6</f>
         <v>46287</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D10" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="33"/>
-      <c r="F8" s="38"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="53" t="s">
+      <c r="E10" s="33"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="62"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="50" t="s">
+      <c r="B11" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="15">
-        <f t="shared" ref="C9" si="1">C7+7</f>
+      <c r="C11" s="15">
+        <f t="shared" ref="C11" si="1">C8+7</f>
         <v>46288</v>
-      </c>
-      <c r="D9" s="18"/>
-      <c r="E9" s="31" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="36"/>
-    </row>
-    <row r="10" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="54"/>
-      <c r="B10" s="52"/>
-      <c r="C10" s="9">
-        <f t="shared" ref="C10" si="2">C9+6</f>
-        <v>46294</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="33"/>
-      <c r="F10" s="38" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="54"/>
-      <c r="B11" s="50" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="15">
-        <f t="shared" ref="C11" si="3">C9+7</f>
-        <v>46295</v>
       </c>
       <c r="D11" s="18"/>
       <c r="E11" s="31" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="36"/>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="54"/>
-      <c r="B12" s="52"/>
+        <v>30</v>
+      </c>
+      <c r="F11" s="54"/>
+      <c r="G11" s="60"/>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="41"/>
+      <c r="B12" s="45"/>
       <c r="C12" s="9">
-        <f t="shared" ref="C12" si="4">C11+6</f>
-        <v>46301</v>
+        <f t="shared" ref="C12" si="2">C11+6</f>
+        <v>46294</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E12" s="33"/>
-      <c r="F12" s="38"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="54"/>
-      <c r="B13" s="50" t="s">
-        <v>6</v>
+      <c r="F12" s="56" t="s">
+        <v>58</v>
+      </c>
+      <c r="G12" s="62"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="41"/>
+      <c r="B13" s="43" t="s">
+        <v>5</v>
       </c>
       <c r="C13" s="15">
-        <f t="shared" ref="C13:C32" si="5">C11+7</f>
-        <v>46302</v>
+        <f t="shared" ref="C13" si="3">C11+7</f>
+        <v>46295</v>
       </c>
       <c r="D13" s="18"/>
       <c r="E13" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="54"/>
+      <c r="G13" s="60"/>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="41"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="9">
+        <f t="shared" ref="C14" si="4">C13+6</f>
+        <v>46301</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="33"/>
+      <c r="F14" s="56"/>
+      <c r="G14" s="62"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="41"/>
+      <c r="B15" s="43" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="15">
+        <f t="shared" ref="C15:C30" si="5">C13+7</f>
+        <v>46302</v>
+      </c>
+      <c r="D15" s="18"/>
+      <c r="E15" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="F13" s="36"/>
-    </row>
-    <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="55"/>
-      <c r="B14" s="52"/>
-      <c r="C14" s="9">
-        <f t="shared" ref="C14:C29" si="6">C13+6</f>
+      <c r="F15" s="54"/>
+      <c r="G15" s="60"/>
+    </row>
+    <row r="16" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="42"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="9">
+        <f t="shared" ref="C16:C29" si="6">C15+6</f>
         <v>46308</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D16" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="E14" s="33"/>
-      <c r="F14" s="38"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="53" t="s">
+      <c r="E16" s="33"/>
+      <c r="F16" s="56"/>
+      <c r="G16" s="62"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="50" t="s">
+      <c r="B17" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="15">
+      <c r="C17" s="15">
         <f t="shared" si="5"/>
         <v>46309</v>
       </c>
-      <c r="D15" s="18"/>
-      <c r="E15" s="31" t="s">
+      <c r="D17" s="18"/>
+      <c r="E17" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="F15" s="36"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="54"/>
-      <c r="B16" s="51"/>
-      <c r="C16" s="3">
+      <c r="F17" s="54"/>
+      <c r="G17" s="60"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="41"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="3">
         <f t="shared" si="6"/>
         <v>46315</v>
       </c>
-      <c r="D16" s="48" t="s">
+      <c r="D18" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="49"/>
-      <c r="F16" s="39"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="54"/>
-      <c r="B17" s="51"/>
-      <c r="C17" s="3">
+      <c r="E18" s="51"/>
+      <c r="F18" s="57"/>
+      <c r="G18" s="61"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="41"/>
+      <c r="B19" s="44"/>
+      <c r="C19" s="3">
         <f t="shared" si="5"/>
         <v>46316</v>
       </c>
-      <c r="D17" s="2"/>
-      <c r="E17" s="32" t="s">
+      <c r="D19" s="2"/>
+      <c r="E19" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="F17" s="37"/>
-    </row>
-    <row r="18" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="54"/>
-      <c r="B18" s="52"/>
-      <c r="C18" s="9">
+      <c r="F19" s="55"/>
+      <c r="G19" s="61"/>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="41"/>
+      <c r="B20" s="45"/>
+      <c r="C20" s="9">
         <f t="shared" si="6"/>
         <v>46322</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D20" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="E18" s="33"/>
-      <c r="F18" s="38" t="s">
+      <c r="E20" s="33"/>
+      <c r="F20" s="56" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="54"/>
-      <c r="B19" s="50" t="s">
+      <c r="G20" s="62"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="41"/>
+      <c r="B21" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="15">
+      <c r="C21" s="15">
         <f t="shared" si="5"/>
         <v>46323</v>
       </c>
-      <c r="D19" s="16"/>
-      <c r="E19" s="31" t="s">
+      <c r="D21" s="16"/>
+      <c r="E21" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="36"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="54"/>
-      <c r="B20" s="51"/>
-      <c r="C20" s="3" t="s">
+      <c r="F21" s="54"/>
+      <c r="G21" s="60"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="41"/>
+      <c r="B22" s="44"/>
+      <c r="C22" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="32"/>
-      <c r="F20" s="37" t="s">
+      <c r="D22" s="2"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="55" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="54"/>
-      <c r="B21" s="52"/>
-      <c r="C21" s="9">
-        <f>C19+6</f>
+      <c r="G22" s="61"/>
+    </row>
+    <row r="23" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="41"/>
+      <c r="B23" s="45"/>
+      <c r="C23" s="9">
+        <f>C21+6</f>
         <v>46329</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="D23" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="38"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="54"/>
-      <c r="B22" s="50" t="s">
+      <c r="E23" s="33"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="62"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="41"/>
+      <c r="B24" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="15">
-        <f>C19+7</f>
+      <c r="C24" s="15">
+        <f>C21+7</f>
         <v>46330</v>
       </c>
-      <c r="D22" s="16"/>
-      <c r="E22" s="31" t="s">
+      <c r="D24" s="16"/>
+      <c r="E24" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="F22" s="36"/>
-    </row>
-    <row r="23" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="55"/>
-      <c r="B23" s="52"/>
-      <c r="C23" s="9">
+      <c r="F24" s="54"/>
+      <c r="G24" s="60"/>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="42"/>
+      <c r="B25" s="45"/>
+      <c r="C25" s="9">
         <f t="shared" si="6"/>
         <v>46336</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D25" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="33"/>
-      <c r="F23" s="38"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="53" t="s">
+      <c r="E25" s="33"/>
+      <c r="F25" s="56"/>
+      <c r="G25" s="62"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="B24" s="50" t="s">
+      <c r="B26" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="15">
+      <c r="C26" s="15">
         <f t="shared" si="5"/>
         <v>46337</v>
       </c>
-      <c r="D24" s="16"/>
-      <c r="E24" s="31" t="s">
+      <c r="D26" s="16"/>
+      <c r="E26" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="F24" s="36" t="s">
+      <c r="F26" s="54" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="54"/>
-      <c r="B25" s="52"/>
-      <c r="C25" s="9">
+      <c r="G26" s="60"/>
+    </row>
+    <row r="27" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="41"/>
+      <c r="B27" s="45"/>
+      <c r="C27" s="9">
         <f t="shared" si="6"/>
         <v>46343</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="D27" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="E25" s="33"/>
-      <c r="F25" s="38"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="54"/>
-      <c r="B26" s="50" t="s">
+      <c r="E27" s="33"/>
+      <c r="F27" s="56"/>
+      <c r="G27" s="62"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="41"/>
+      <c r="B28" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="C26" s="15">
+      <c r="C28" s="15">
         <f t="shared" si="5"/>
         <v>46344</v>
       </c>
-      <c r="D26" s="16"/>
-      <c r="E26" s="31" t="s">
+      <c r="D28" s="16"/>
+      <c r="E28" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="F26" s="36"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="54"/>
-      <c r="B27" s="51"/>
-      <c r="C27" s="3">
+      <c r="F28" s="54"/>
+      <c r="G28" s="60"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="41"/>
+      <c r="B29" s="44"/>
+      <c r="C29" s="3">
         <f t="shared" si="6"/>
         <v>46350</v>
       </c>
-      <c r="D27" s="1"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="37"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="54"/>
-      <c r="B28" s="51"/>
-      <c r="C28" s="3">
+      <c r="D29" s="1"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="55"/>
+      <c r="G29" s="61"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="41"/>
+      <c r="B30" s="44"/>
+      <c r="C30" s="3">
         <f t="shared" si="5"/>
         <v>46351</v>
       </c>
-      <c r="D28" s="48" t="s">
+      <c r="D30" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="E28" s="49"/>
-      <c r="F28" s="39"/>
-    </row>
-    <row r="29" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="54"/>
-      <c r="B29" s="52"/>
-      <c r="C29" s="9">
-        <f t="shared" si="6"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="57"/>
+      <c r="G30" s="61"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="41"/>
+      <c r="B31" s="44"/>
+      <c r="C31" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" s="38"/>
+      <c r="E31" s="39"/>
+      <c r="F31" s="57"/>
+      <c r="G31" s="61" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="41"/>
+      <c r="B32" s="45"/>
+      <c r="C32" s="9">
+        <f>C30+6</f>
         <v>46357</v>
       </c>
-      <c r="D29" s="17" t="s">
+      <c r="D32" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="E29" s="33"/>
-      <c r="F29" s="38"/>
-    </row>
-    <row r="30" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="54"/>
-      <c r="B30" s="50" t="s">
+      <c r="E32" s="33"/>
+      <c r="F32" s="56"/>
+      <c r="G32" s="62"/>
+    </row>
+    <row r="33" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="41"/>
+      <c r="B33" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="C30" s="15">
-        <f t="shared" si="5"/>
+      <c r="C33" s="15">
+        <f>C30+7</f>
         <v>46358</v>
       </c>
-      <c r="D30" s="19"/>
-      <c r="E30" s="31" t="s">
+      <c r="D33" s="19"/>
+      <c r="E33" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="F30" s="40"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="54"/>
-      <c r="B31" s="51"/>
-      <c r="C31" s="3">
-        <f>C30+1</f>
+      <c r="F33" s="58"/>
+      <c r="G33" s="63"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A34" s="41"/>
+      <c r="B34" s="44"/>
+      <c r="C34" s="3">
+        <f>C33+1</f>
         <v>46359</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D34" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E31" s="32"/>
-      <c r="F31" s="37"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="54"/>
-      <c r="B32" s="51"/>
-      <c r="C32" s="3">
-        <f t="shared" si="5"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="55"/>
+      <c r="G34" s="61"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A35" s="41"/>
+      <c r="B35" s="44"/>
+      <c r="C35" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D35" s="2"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="55"/>
+      <c r="G35" s="61" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" s="41"/>
+      <c r="B36" s="44"/>
+      <c r="C36" s="3">
+        <f>C33+7</f>
         <v>46365</v>
       </c>
-      <c r="D32" s="1"/>
-      <c r="E32" s="32" t="s">
+      <c r="D36" s="1"/>
+      <c r="E36" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F32" s="37"/>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="54"/>
-      <c r="B33" s="51"/>
-      <c r="C33" s="3">
-        <f>C32+2</f>
+      <c r="F36" s="55"/>
+      <c r="G36" s="61"/>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A37" s="41"/>
+      <c r="B37" s="44"/>
+      <c r="C37" s="3">
+        <f>C36+2</f>
         <v>46367</v>
       </c>
-      <c r="D33" s="41"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="37"/>
-    </row>
-    <row r="34" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="55"/>
-      <c r="B34" s="52"/>
-      <c r="C34" s="9">
+      <c r="D37" s="36"/>
+      <c r="E37" s="34"/>
+      <c r="F37" s="55"/>
+      <c r="G37" s="61"/>
+    </row>
+    <row r="38" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="42"/>
+      <c r="B38" s="45"/>
+      <c r="C38" s="9">
         <v>46375</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="D38" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E34" s="35"/>
-      <c r="F34" s="42"/>
-    </row>
-    <row r="35" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="36" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="20" t="s">
+      <c r="E38" s="35"/>
+      <c r="F38" s="59"/>
+      <c r="G38" s="62"/>
+    </row>
+    <row r="39" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="21"/>
-      <c r="C36" s="22"/>
-      <c r="D36" s="23"/>
-      <c r="E36" s="23"/>
-      <c r="F36" s="21"/>
-      <c r="G36" s="24"/>
-      <c r="H36" s="24"/>
-      <c r="I36" s="24"/>
-      <c r="J36" s="24"/>
-      <c r="K36" s="24"/>
-      <c r="L36" s="24"/>
-      <c r="M36" s="24"/>
-      <c r="N36" s="24"/>
-      <c r="O36" s="25"/>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" s="26"/>
-      <c r="O37" s="27"/>
-    </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A38" s="26"/>
-      <c r="B38" t="s">
+      <c r="B40" s="21"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="23"/>
+      <c r="E40" s="23"/>
+      <c r="F40" s="21"/>
+      <c r="G40" s="24"/>
+      <c r="H40" s="24"/>
+      <c r="I40" s="24"/>
+      <c r="J40" s="24"/>
+      <c r="K40" s="24"/>
+      <c r="L40" s="24"/>
+      <c r="M40" s="24"/>
+      <c r="N40" s="24"/>
+      <c r="O40" s="25"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A41" s="26"/>
+      <c r="O41" s="27"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A42" s="26"/>
+      <c r="B42" t="s">
         <v>50</v>
       </c>
-      <c r="C38" s="44" t="s">
+      <c r="C42" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="D38" s="44"/>
-      <c r="E38" s="44"/>
-      <c r="F38" s="44"/>
-      <c r="G38" s="44"/>
-      <c r="H38" s="44"/>
-      <c r="I38" s="44"/>
-      <c r="J38" s="44"/>
-      <c r="K38" s="44"/>
-      <c r="L38" s="44"/>
-      <c r="M38" s="44"/>
-      <c r="N38" s="44"/>
-      <c r="O38" s="45"/>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A39" s="26"/>
-      <c r="B39" t="s">
+      <c r="D42" s="46"/>
+      <c r="E42" s="46"/>
+      <c r="F42" s="46"/>
+      <c r="G42" s="46"/>
+      <c r="H42" s="46"/>
+      <c r="I42" s="46"/>
+      <c r="J42" s="46"/>
+      <c r="K42" s="46"/>
+      <c r="L42" s="46"/>
+      <c r="M42" s="46"/>
+      <c r="N42" s="46"/>
+      <c r="O42" s="47"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" s="26"/>
+      <c r="B43" t="s">
         <v>51</v>
       </c>
-      <c r="C39" s="44" t="s">
+      <c r="C43" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="D39" s="44"/>
-      <c r="E39" s="44"/>
-      <c r="F39" s="44"/>
-      <c r="G39" s="44"/>
-      <c r="H39" s="44"/>
-      <c r="I39" s="44"/>
-      <c r="J39" s="44"/>
-      <c r="K39" s="44"/>
-      <c r="L39" s="44"/>
-      <c r="M39" s="44"/>
-      <c r="N39" s="44"/>
-      <c r="O39" s="45"/>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A40" s="26"/>
-      <c r="B40" t="s">
+      <c r="D43" s="46"/>
+      <c r="E43" s="46"/>
+      <c r="F43" s="46"/>
+      <c r="G43" s="46"/>
+      <c r="H43" s="46"/>
+      <c r="I43" s="46"/>
+      <c r="J43" s="46"/>
+      <c r="K43" s="46"/>
+      <c r="L43" s="46"/>
+      <c r="M43" s="46"/>
+      <c r="N43" s="46"/>
+      <c r="O43" s="47"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" s="26"/>
+      <c r="B44" t="s">
         <v>52</v>
       </c>
-      <c r="C40" s="44" t="s">
+      <c r="C44" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="D40" s="44"/>
-      <c r="E40" s="44"/>
-      <c r="F40" s="44"/>
-      <c r="G40" s="44"/>
-      <c r="H40" s="44"/>
-      <c r="I40" s="44"/>
-      <c r="J40" s="44"/>
-      <c r="K40" s="44"/>
-      <c r="L40" s="44"/>
-      <c r="M40" s="44"/>
-      <c r="N40" s="44"/>
-      <c r="O40" s="45"/>
-    </row>
-    <row r="41" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="28"/>
-      <c r="B41" s="29" t="s">
+      <c r="D44" s="46"/>
+      <c r="E44" s="46"/>
+      <c r="F44" s="46"/>
+      <c r="G44" s="46"/>
+      <c r="H44" s="46"/>
+      <c r="I44" s="46"/>
+      <c r="J44" s="46"/>
+      <c r="K44" s="46"/>
+      <c r="L44" s="46"/>
+      <c r="M44" s="46"/>
+      <c r="N44" s="46"/>
+      <c r="O44" s="47"/>
+    </row>
+    <row r="45" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="28"/>
+      <c r="B45" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="C41" s="46" t="s">
+      <c r="C45" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="D41" s="46"/>
-      <c r="E41" s="46"/>
-      <c r="F41" s="46"/>
-      <c r="G41" s="46"/>
-      <c r="H41" s="46"/>
-      <c r="I41" s="46"/>
-      <c r="J41" s="46"/>
-      <c r="K41" s="46"/>
-      <c r="L41" s="46"/>
-      <c r="M41" s="46"/>
-      <c r="N41" s="46"/>
-      <c r="O41" s="47"/>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B42"/>
-      <c r="C42"/>
-      <c r="D42"/>
-      <c r="E42"/>
-      <c r="F42"/>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>63</v>
-      </c>
-      <c r="B43"/>
-      <c r="C43"/>
-      <c r="D43"/>
-      <c r="E43"/>
-      <c r="F43"/>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B44"/>
-      <c r="C44"/>
-      <c r="D44"/>
-      <c r="E44"/>
-      <c r="F44"/>
-    </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B45"/>
-      <c r="C45"/>
-      <c r="D45"/>
-      <c r="E45"/>
-      <c r="F45"/>
+      <c r="D45" s="48"/>
+      <c r="E45" s="48"/>
+      <c r="F45" s="48"/>
+      <c r="G45" s="48"/>
+      <c r="H45" s="48"/>
+      <c r="I45" s="48"/>
+      <c r="J45" s="48"/>
+      <c r="K45" s="48"/>
+      <c r="L45" s="48"/>
+      <c r="M45" s="48"/>
+      <c r="N45" s="48"/>
+      <c r="O45" s="49"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B46"/>
@@ -1747,6 +1870,9 @@
       <c r="F46"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>63</v>
+      </c>
       <c r="B47"/>
       <c r="C47"/>
       <c r="D47"/>
@@ -1766,30 +1892,34 @@
     <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A2:A8"/>
-    <mergeCell ref="A9:A14"/>
-    <mergeCell ref="A15:A23"/>
-    <mergeCell ref="A24:A34"/>
+    <mergeCell ref="C44:O44"/>
+    <mergeCell ref="C45:O45"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="B33:B38"/>
+    <mergeCell ref="C42:O42"/>
+    <mergeCell ref="C43:O43"/>
+    <mergeCell ref="A2:A10"/>
+    <mergeCell ref="A11:A16"/>
+    <mergeCell ref="A17:A25"/>
+    <mergeCell ref="A26:A38"/>
     <mergeCell ref="B2:B4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
     <mergeCell ref="B11:B12"/>
     <mergeCell ref="B13:B14"/>
-    <mergeCell ref="B15:B18"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="B21:B23"/>
     <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="C40:O40"/>
-    <mergeCell ref="C41:O41"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="B30:B34"/>
-    <mergeCell ref="C38:O38"/>
-    <mergeCell ref="C39:O39"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B28:B32"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: update chalk talk schedule and link version in index
</commit_message>
<xml_diff>
--- a/comp560-schedule.xlsx
+++ b/comp560-schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp560-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CBB5306-000C-4F94-99C9-17D012E37D27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DEAEDB-96F2-40A3-957D-1BEB8992B710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -224,9 +224,6 @@
     <t>Priestley Award</t>
   </si>
   <si>
-    <t>updated 9/2/2026</t>
-  </si>
-  <si>
     <t>honors projects</t>
   </si>
   <si>
@@ -252,6 +249,9 @@
   </si>
   <si>
     <t>complete draft of RR</t>
+  </si>
+  <si>
+    <t>updated 9/9/2026</t>
   </si>
 </sst>
 </file>
@@ -262,7 +262,7 @@
     <numFmt numFmtId="164" formatCode="m/d;@"/>
     <numFmt numFmtId="165" formatCode="ddd\ m/d"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -305,6 +305,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -708,7 +716,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -811,45 +819,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -875,6 +844,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1207,18 +1218,18 @@
       <c r="E1" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="53" t="s">
+      <c r="F1" s="40" t="s">
         <v>59</v>
       </c>
       <c r="G1" s="37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="57" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="15">
@@ -1226,12 +1237,12 @@
       </c>
       <c r="D2" s="16"/>
       <c r="E2" s="31"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="60"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="47"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="41"/>
-      <c r="B3" s="44"/>
+      <c r="A3" s="61"/>
+      <c r="B3" s="58"/>
       <c r="C3" s="3">
         <v>46267</v>
       </c>
@@ -1239,12 +1250,12 @@
       <c r="E3" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="55"/>
-      <c r="G3" s="61"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="48"/>
     </row>
     <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="41"/>
-      <c r="B4" s="45"/>
+      <c r="A4" s="61"/>
+      <c r="B4" s="59"/>
       <c r="C4" s="9">
         <v>46273</v>
       </c>
@@ -1252,12 +1263,12 @@
         <v>17</v>
       </c>
       <c r="E4" s="33"/>
-      <c r="F4" s="56"/>
-      <c r="G4" s="62"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="49"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="41"/>
-      <c r="B5" s="43" t="s">
+      <c r="A5" s="61"/>
+      <c r="B5" s="57" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="15">
@@ -1267,25 +1278,25 @@
       <c r="E5" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="54"/>
-      <c r="G5" s="60"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="47"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="41"/>
-      <c r="B6" s="44"/>
+      <c r="A6" s="61"/>
+      <c r="B6" s="58"/>
       <c r="C6" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="32"/>
-      <c r="F6" s="55"/>
-      <c r="G6" s="61" t="s">
-        <v>71</v>
+      <c r="F6" s="42"/>
+      <c r="G6" s="48" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="41"/>
-      <c r="B7" s="45"/>
+      <c r="A7" s="61"/>
+      <c r="B7" s="59"/>
       <c r="C7" s="9">
         <f>C5+6</f>
         <v>46280</v>
@@ -1294,12 +1305,12 @@
         <v>18</v>
       </c>
       <c r="E7" s="33"/>
-      <c r="F7" s="56"/>
-      <c r="G7" s="62"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="49"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="41"/>
-      <c r="B8" s="43" t="s">
+      <c r="A8" s="61"/>
+      <c r="B8" s="57" t="s">
         <v>3</v>
       </c>
       <c r="C8" s="15">
@@ -1310,25 +1321,25 @@
       <c r="E8" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="54"/>
-      <c r="G8" s="60"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="47"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="52"/>
-      <c r="B9" s="44"/>
+      <c r="A9" s="62"/>
+      <c r="B9" s="58"/>
       <c r="C9" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="32"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="61" t="s">
-        <v>66</v>
+      <c r="F9" s="42"/>
+      <c r="G9" s="48" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="42"/>
-      <c r="B10" s="45"/>
+      <c r="A10" s="63"/>
+      <c r="B10" s="59"/>
       <c r="C10" s="9">
         <f t="shared" ref="C10" si="0">C8+6</f>
         <v>46287</v>
@@ -1337,14 +1348,14 @@
         <v>45</v>
       </c>
       <c r="E10" s="33"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="62"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="49"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="40" t="s">
+      <c r="A11" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="43" t="s">
+      <c r="B11" s="57" t="s">
         <v>4</v>
       </c>
       <c r="C11" s="15">
@@ -1355,12 +1366,12 @@
       <c r="E11" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="54"/>
-      <c r="G11" s="60"/>
+      <c r="F11" s="41"/>
+      <c r="G11" s="47"/>
     </row>
     <row r="12" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="41"/>
-      <c r="B12" s="45"/>
+      <c r="A12" s="61"/>
+      <c r="B12" s="59"/>
       <c r="C12" s="9">
         <f t="shared" ref="C12" si="2">C11+6</f>
         <v>46294</v>
@@ -1369,14 +1380,14 @@
         <v>19</v>
       </c>
       <c r="E12" s="33"/>
-      <c r="F12" s="56" t="s">
+      <c r="F12" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="G12" s="62"/>
+      <c r="G12" s="49"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="41"/>
-      <c r="B13" s="43" t="s">
+      <c r="A13" s="61"/>
+      <c r="B13" s="57" t="s">
         <v>5</v>
       </c>
       <c r="C13" s="15">
@@ -1387,12 +1398,12 @@
       <c r="E13" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="F13" s="54"/>
-      <c r="G13" s="60"/>
+      <c r="F13" s="41"/>
+      <c r="G13" s="47"/>
     </row>
     <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="41"/>
-      <c r="B14" s="45"/>
+      <c r="A14" s="61"/>
+      <c r="B14" s="59"/>
       <c r="C14" s="9">
         <f t="shared" ref="C14" si="4">C13+6</f>
         <v>46301</v>
@@ -1401,12 +1412,12 @@
         <v>20</v>
       </c>
       <c r="E14" s="33"/>
-      <c r="F14" s="56"/>
-      <c r="G14" s="62"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="49"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="41"/>
-      <c r="B15" s="43" t="s">
+      <c r="A15" s="61"/>
+      <c r="B15" s="57" t="s">
         <v>6</v>
       </c>
       <c r="C15" s="15">
@@ -1417,12 +1428,12 @@
       <c r="E15" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="54"/>
-      <c r="G15" s="60"/>
+      <c r="F15" s="41"/>
+      <c r="G15" s="47"/>
     </row>
     <row r="16" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="42"/>
-      <c r="B16" s="45"/>
+      <c r="A16" s="63"/>
+      <c r="B16" s="59"/>
       <c r="C16" s="9">
         <f t="shared" ref="C16:C29" si="6">C15+6</f>
         <v>46308</v>
@@ -1431,14 +1442,14 @@
         <v>46</v>
       </c>
       <c r="E16" s="33"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="62"/>
+      <c r="F16" s="43"/>
+      <c r="G16" s="49"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="43" t="s">
+      <c r="B17" s="57" t="s">
         <v>7</v>
       </c>
       <c r="C17" s="15">
@@ -1449,26 +1460,26 @@
       <c r="E17" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="F17" s="54"/>
-      <c r="G17" s="60"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="47"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="41"/>
-      <c r="B18" s="44"/>
+      <c r="A18" s="61"/>
+      <c r="B18" s="58"/>
       <c r="C18" s="3">
         <f t="shared" si="6"/>
         <v>46315</v>
       </c>
-      <c r="D18" s="50" t="s">
+      <c r="D18" s="55" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="51"/>
-      <c r="F18" s="57"/>
-      <c r="G18" s="61"/>
+      <c r="E18" s="56"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="48"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="41"/>
-      <c r="B19" s="44"/>
+      <c r="A19" s="61"/>
+      <c r="B19" s="58"/>
       <c r="C19" s="3">
         <f t="shared" si="5"/>
         <v>46316</v>
@@ -1477,12 +1488,12 @@
       <c r="E19" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="F19" s="55"/>
-      <c r="G19" s="61"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="48"/>
     </row>
     <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="41"/>
-      <c r="B20" s="45"/>
+      <c r="A20" s="61"/>
+      <c r="B20" s="59"/>
       <c r="C20" s="9">
         <f t="shared" si="6"/>
         <v>46322</v>
@@ -1491,14 +1502,14 @@
         <v>21</v>
       </c>
       <c r="E20" s="33"/>
-      <c r="F20" s="56" t="s">
+      <c r="F20" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="G20" s="62"/>
+      <c r="G20" s="49"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="41"/>
-      <c r="B21" s="43" t="s">
+      <c r="A21" s="61"/>
+      <c r="B21" s="57" t="s">
         <v>8</v>
       </c>
       <c r="C21" s="15">
@@ -1509,25 +1520,25 @@
       <c r="E21" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="F21" s="54"/>
-      <c r="G21" s="60"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="47"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="41"/>
-      <c r="B22" s="44"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="58"/>
       <c r="C22" s="3" t="s">
         <v>52</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="32"/>
-      <c r="F22" s="55" t="s">
+      <c r="F22" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="G22" s="61"/>
+      <c r="G22" s="48"/>
     </row>
     <row r="23" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="41"/>
-      <c r="B23" s="45"/>
+      <c r="A23" s="61"/>
+      <c r="B23" s="59"/>
       <c r="C23" s="9">
         <f>C21+6</f>
         <v>46329</v>
@@ -1536,12 +1547,12 @@
         <v>22</v>
       </c>
       <c r="E23" s="33"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="62"/>
+      <c r="F23" s="43"/>
+      <c r="G23" s="49"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="41"/>
-      <c r="B24" s="43" t="s">
+      <c r="A24" s="61"/>
+      <c r="B24" s="57" t="s">
         <v>9</v>
       </c>
       <c r="C24" s="15">
@@ -1552,12 +1563,12 @@
       <c r="E24" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="F24" s="54"/>
-      <c r="G24" s="60"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="47"/>
     </row>
     <row r="25" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="42"/>
-      <c r="B25" s="45"/>
+      <c r="A25" s="63"/>
+      <c r="B25" s="59"/>
       <c r="C25" s="9">
         <f t="shared" si="6"/>
         <v>46336</v>
@@ -1566,14 +1577,14 @@
         <v>47</v>
       </c>
       <c r="E25" s="33"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="62"/>
+      <c r="F25" s="43"/>
+      <c r="G25" s="49"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="40" t="s">
+      <c r="A26" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="B26" s="43" t="s">
+      <c r="B26" s="57" t="s">
         <v>10</v>
       </c>
       <c r="C26" s="15">
@@ -1581,17 +1592,17 @@
         <v>46337</v>
       </c>
       <c r="D26" s="16"/>
-      <c r="E26" s="31" t="s">
+      <c r="E26" s="64" t="s">
         <v>35</v>
       </c>
-      <c r="F26" s="54" t="s">
+      <c r="F26" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="G26" s="60"/>
+      <c r="G26" s="47"/>
     </row>
     <row r="27" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="41"/>
-      <c r="B27" s="45"/>
+      <c r="A27" s="61"/>
+      <c r="B27" s="59"/>
       <c r="C27" s="9">
         <f t="shared" si="6"/>
         <v>46343</v>
@@ -1600,12 +1611,12 @@
         <v>23</v>
       </c>
       <c r="E27" s="33"/>
-      <c r="F27" s="56"/>
-      <c r="G27" s="62"/>
+      <c r="F27" s="43"/>
+      <c r="G27" s="49"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="41"/>
-      <c r="B28" s="43" t="s">
+      <c r="A28" s="61"/>
+      <c r="B28" s="57" t="s">
         <v>11</v>
       </c>
       <c r="C28" s="15">
@@ -1616,51 +1627,51 @@
       <c r="E28" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="F28" s="54"/>
-      <c r="G28" s="60"/>
+      <c r="F28" s="41"/>
+      <c r="G28" s="47"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="41"/>
-      <c r="B29" s="44"/>
+      <c r="A29" s="61"/>
+      <c r="B29" s="58"/>
       <c r="C29" s="3">
         <f t="shared" si="6"/>
         <v>46350</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="32"/>
-      <c r="F29" s="55"/>
-      <c r="G29" s="61"/>
+      <c r="F29" s="42"/>
+      <c r="G29" s="48"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="41"/>
-      <c r="B30" s="44"/>
+      <c r="A30" s="61"/>
+      <c r="B30" s="58"/>
       <c r="C30" s="3">
         <f t="shared" si="5"/>
         <v>46351</v>
       </c>
-      <c r="D30" s="50" t="s">
+      <c r="D30" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="E30" s="51"/>
-      <c r="F30" s="57"/>
-      <c r="G30" s="61"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="44"/>
+      <c r="G30" s="48"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="41"/>
-      <c r="B31" s="44"/>
+      <c r="A31" s="61"/>
+      <c r="B31" s="58"/>
       <c r="C31" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D31" s="38"/>
       <c r="E31" s="39"/>
-      <c r="F31" s="57"/>
-      <c r="G31" s="61" t="s">
-        <v>72</v>
+      <c r="F31" s="44"/>
+      <c r="G31" s="48" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="41"/>
-      <c r="B32" s="45"/>
+      <c r="A32" s="61"/>
+      <c r="B32" s="59"/>
       <c r="C32" s="9">
         <f>C30+6</f>
         <v>46357</v>
@@ -1669,12 +1680,12 @@
         <v>24</v>
       </c>
       <c r="E32" s="33"/>
-      <c r="F32" s="56"/>
-      <c r="G32" s="62"/>
+      <c r="F32" s="43"/>
+      <c r="G32" s="49"/>
     </row>
     <row r="33" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="41"/>
-      <c r="B33" s="43" t="s">
+      <c r="A33" s="61"/>
+      <c r="B33" s="57" t="s">
         <v>12</v>
       </c>
       <c r="C33" s="15">
@@ -1685,12 +1696,12 @@
       <c r="E33" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="F33" s="58"/>
-      <c r="G33" s="63"/>
+      <c r="F33" s="45"/>
+      <c r="G33" s="50"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A34" s="41"/>
-      <c r="B34" s="44"/>
+      <c r="A34" s="61"/>
+      <c r="B34" s="58"/>
       <c r="C34" s="3">
         <f>C33+1</f>
         <v>46359</v>
@@ -1699,25 +1710,25 @@
         <v>25</v>
       </c>
       <c r="E34" s="32"/>
-      <c r="F34" s="55"/>
-      <c r="G34" s="61"/>
+      <c r="F34" s="42"/>
+      <c r="G34" s="48"/>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="41"/>
-      <c r="B35" s="44"/>
+      <c r="A35" s="61"/>
+      <c r="B35" s="58"/>
       <c r="C35" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="32"/>
-      <c r="F35" s="55"/>
-      <c r="G35" s="61" t="s">
-        <v>69</v>
+      <c r="F35" s="42"/>
+      <c r="G35" s="48" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A36" s="41"/>
-      <c r="B36" s="44"/>
+      <c r="A36" s="61"/>
+      <c r="B36" s="58"/>
       <c r="C36" s="3">
         <f>C33+7</f>
         <v>46365</v>
@@ -1726,24 +1737,24 @@
       <c r="E36" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F36" s="55"/>
-      <c r="G36" s="61"/>
+      <c r="F36" s="42"/>
+      <c r="G36" s="48"/>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" s="41"/>
-      <c r="B37" s="44"/>
+      <c r="A37" s="61"/>
+      <c r="B37" s="58"/>
       <c r="C37" s="3">
         <f>C36+2</f>
         <v>46367</v>
       </c>
       <c r="D37" s="36"/>
       <c r="E37" s="34"/>
-      <c r="F37" s="55"/>
-      <c r="G37" s="61"/>
+      <c r="F37" s="42"/>
+      <c r="G37" s="48"/>
     </row>
     <row r="38" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="42"/>
-      <c r="B38" s="45"/>
+      <c r="A38" s="63"/>
+      <c r="B38" s="59"/>
       <c r="C38" s="9">
         <v>46375</v>
       </c>
@@ -1751,8 +1762,8 @@
         <v>48</v>
       </c>
       <c r="E38" s="35"/>
-      <c r="F38" s="59"/>
-      <c r="G38" s="62"/>
+      <c r="F38" s="46"/>
+      <c r="G38" s="49"/>
     </row>
     <row r="39" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="40" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
@@ -1783,84 +1794,84 @@
       <c r="B42" t="s">
         <v>50</v>
       </c>
-      <c r="C42" s="46" t="s">
+      <c r="C42" s="51" t="s">
         <v>54</v>
       </c>
-      <c r="D42" s="46"/>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46"/>
-      <c r="H42" s="46"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="46"/>
-      <c r="K42" s="46"/>
-      <c r="L42" s="46"/>
-      <c r="M42" s="46"/>
-      <c r="N42" s="46"/>
-      <c r="O42" s="47"/>
+      <c r="D42" s="51"/>
+      <c r="E42" s="51"/>
+      <c r="F42" s="51"/>
+      <c r="G42" s="51"/>
+      <c r="H42" s="51"/>
+      <c r="I42" s="51"/>
+      <c r="J42" s="51"/>
+      <c r="K42" s="51"/>
+      <c r="L42" s="51"/>
+      <c r="M42" s="51"/>
+      <c r="N42" s="51"/>
+      <c r="O42" s="52"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="26"/>
       <c r="B43" t="s">
         <v>51</v>
       </c>
-      <c r="C43" s="46" t="s">
+      <c r="C43" s="51" t="s">
         <v>55</v>
       </c>
-      <c r="D43" s="46"/>
-      <c r="E43" s="46"/>
-      <c r="F43" s="46"/>
-      <c r="G43" s="46"/>
-      <c r="H43" s="46"/>
-      <c r="I43" s="46"/>
-      <c r="J43" s="46"/>
-      <c r="K43" s="46"/>
-      <c r="L43" s="46"/>
-      <c r="M43" s="46"/>
-      <c r="N43" s="46"/>
-      <c r="O43" s="47"/>
+      <c r="D43" s="51"/>
+      <c r="E43" s="51"/>
+      <c r="F43" s="51"/>
+      <c r="G43" s="51"/>
+      <c r="H43" s="51"/>
+      <c r="I43" s="51"/>
+      <c r="J43" s="51"/>
+      <c r="K43" s="51"/>
+      <c r="L43" s="51"/>
+      <c r="M43" s="51"/>
+      <c r="N43" s="51"/>
+      <c r="O43" s="52"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="26"/>
       <c r="B44" t="s">
         <v>52</v>
       </c>
-      <c r="C44" s="46" t="s">
+      <c r="C44" s="51" t="s">
         <v>56</v>
       </c>
-      <c r="D44" s="46"/>
-      <c r="E44" s="46"/>
-      <c r="F44" s="46"/>
-      <c r="G44" s="46"/>
-      <c r="H44" s="46"/>
-      <c r="I44" s="46"/>
-      <c r="J44" s="46"/>
-      <c r="K44" s="46"/>
-      <c r="L44" s="46"/>
-      <c r="M44" s="46"/>
-      <c r="N44" s="46"/>
-      <c r="O44" s="47"/>
+      <c r="D44" s="51"/>
+      <c r="E44" s="51"/>
+      <c r="F44" s="51"/>
+      <c r="G44" s="51"/>
+      <c r="H44" s="51"/>
+      <c r="I44" s="51"/>
+      <c r="J44" s="51"/>
+      <c r="K44" s="51"/>
+      <c r="L44" s="51"/>
+      <c r="M44" s="51"/>
+      <c r="N44" s="51"/>
+      <c r="O44" s="52"/>
     </row>
     <row r="45" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="28"/>
       <c r="B45" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="C45" s="48" t="s">
+      <c r="C45" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="D45" s="48"/>
-      <c r="E45" s="48"/>
-      <c r="F45" s="48"/>
-      <c r="G45" s="48"/>
-      <c r="H45" s="48"/>
-      <c r="I45" s="48"/>
-      <c r="J45" s="48"/>
-      <c r="K45" s="48"/>
-      <c r="L45" s="48"/>
-      <c r="M45" s="48"/>
-      <c r="N45" s="48"/>
-      <c r="O45" s="49"/>
+      <c r="D45" s="53"/>
+      <c r="E45" s="53"/>
+      <c r="F45" s="53"/>
+      <c r="G45" s="53"/>
+      <c r="H45" s="53"/>
+      <c r="I45" s="53"/>
+      <c r="J45" s="53"/>
+      <c r="K45" s="53"/>
+      <c r="L45" s="53"/>
+      <c r="M45" s="53"/>
+      <c r="N45" s="53"/>
+      <c r="O45" s="54"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B46"/>
@@ -1871,7 +1882,7 @@
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="B47"/>
       <c r="C47"/>
@@ -1898,13 +1909,6 @@
     <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C44:O44"/>
-    <mergeCell ref="C45:O45"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="B33:B38"/>
-    <mergeCell ref="C42:O42"/>
-    <mergeCell ref="C43:O43"/>
     <mergeCell ref="A2:A10"/>
     <mergeCell ref="A11:A16"/>
     <mergeCell ref="A17:A25"/>
@@ -1920,9 +1924,16 @@
     <mergeCell ref="B24:B25"/>
     <mergeCell ref="B26:B27"/>
     <mergeCell ref="B28:B32"/>
+    <mergeCell ref="C44:O44"/>
+    <mergeCell ref="C45:O45"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="B33:B38"/>
+    <mergeCell ref="C42:O42"/>
+    <mergeCell ref="C43:O43"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="51" fitToHeight="0" orientation="landscape" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup scale="51" fitToHeight="0" orientation="landscape" horizontalDpi="4294967293" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>